<commit_message>
Created ThreadLocal class to avoid data conflicts in parallel execution
</commit_message>
<xml_diff>
--- a/testData/OpenCart_LoginData1.xlsx
+++ b/testData/OpenCart_LoginData1.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="23">
   <si>
     <t>username</t>
   </si>
@@ -67,6 +67,45 @@
   </si>
   <si>
     <t>JjjMm</t>
+  </si>
+  <si>
+    <t>HxvJr</t>
+  </si>
+  <si>
+    <t>Zisqu</t>
+  </si>
+  <si>
+    <t>CnVwO</t>
+  </si>
+  <si>
+    <t>QfWNj</t>
+  </si>
+  <si>
+    <t>OLbAF</t>
+  </si>
+  <si>
+    <t>IhNbo</t>
+  </si>
+  <si>
+    <t>ZHXRq</t>
+  </si>
+  <si>
+    <t>ybWML</t>
+  </si>
+  <si>
+    <t>xZnTq</t>
+  </si>
+  <si>
+    <t>CLumq</t>
+  </si>
+  <si>
+    <t>eNLat</t>
+  </si>
+  <si>
+    <t>cfKOU</t>
+  </si>
+  <si>
+    <t>DjdVC</t>
   </si>
 </sst>
 </file>
@@ -435,10 +474,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>3</v>
@@ -446,10 +485,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s" s="0">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s" s="0">
         <v>3</v>
@@ -457,10 +496,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s" s="0">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s" s="0">
         <v>3</v>

</xml_diff>